<commit_message>
MAJ ressources FHIR d9324e9e7a21f34b27f7befd64591c3181960c35
</commit_message>
<xml_diff>
--- a/htr-corps-ressources-FHIR/ig/StructureDefinition-fr-actor-extension.xlsx
+++ b/htr-corps-ressources-FHIR/ig/StructureDefinition-fr-actor-extension.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="138">
   <si>
     <t>Property</t>
   </si>
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Fr Extension - Actor</t>
+    <t>Extension - Actor</t>
   </si>
   <si>
     <t>Status</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-09-01T13:19:09+00:00</t>
+    <t>2025-09-02T15:19:36+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -129,7 +129,7 @@
     <t>Context</t>
   </si>
   <si>
-    <t>element:Resource</t>
+    <t>element:Element</t>
   </si>
   <si>
     <t>ID</t>
@@ -387,6 +387,31 @@
 </t>
   </si>
   <si>
+    <t>Extension.extension:typeCode</t>
+  </si>
+  <si>
+    <t>typeCode</t>
+  </si>
+  <si>
+    <t>Type de participation</t>
+  </si>
+  <si>
+    <t>Extension.extension:typeCode.id</t>
+  </si>
+  <si>
+    <t>Extension.extension:typeCode.extension</t>
+  </si>
+  <si>
+    <t>Extension.extension:typeCode.url</t>
+  </si>
+  <si>
+    <t>Extension.extension:typeCode.value[x]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CodeableConcept
+</t>
+  </si>
+  <si>
     <t>Extension.extension:reference</t>
   </si>
   <si>
@@ -408,7 +433,7 @@
     <t>Extension.extension:reference.value[x]</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-practitionerRole-document)
+    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-practitionerRole-document|Device|https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-device-document|https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-organization-document|https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-related-person-document|https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-patient-ins-document|https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-patient-document)
 </t>
   </si>
   <si>
@@ -723,7 +748,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK16"/>
+  <dimension ref="A1:AK21"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="33.09375" customWidth="true" bestFit="true"/>
@@ -1718,7 +1743,7 @@
       </c>
       <c r="E10" s="2"/>
       <c r="F10" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="G10" t="s" s="2">
         <v>83</v>
@@ -2224,12 +2249,14 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="C15" s="2"/>
+        <v>89</v>
+      </c>
+      <c r="C15" t="s" s="2">
+        <v>130</v>
+      </c>
       <c r="D15" t="s" s="2">
         <v>76</v>
       </c>
@@ -2250,24 +2277,22 @@
         <v>76</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>106</v>
+        <v>91</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>107</v>
+        <v>131</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>108</v>
-      </c>
-      <c r="N15" t="s" s="2">
-        <v>109</v>
-      </c>
+        <v>92</v>
+      </c>
+      <c r="N15" s="2"/>
       <c r="O15" s="2"/>
       <c r="P15" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q15" s="2"/>
       <c r="R15" t="s" s="2">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="S15" t="s" s="2">
         <v>76</v>
@@ -2309,30 +2334,30 @@
         <v>76</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="AG15" t="s" s="2">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="AH15" t="s" s="2">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="AI15" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ15" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AK15" t="s" s="2">
-        <v>111</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2343,7 +2368,7 @@
         <v>77</v>
       </c>
       <c r="G16" t="s" s="2">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H16" t="s" s="2">
         <v>76</v>
@@ -2355,13 +2380,13 @@
         <v>76</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>129</v>
+        <v>84</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>116</v>
+        <v>86</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -2412,21 +2437,540 @@
         <v>76</v>
       </c>
       <c r="AF16" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="AG16" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH16" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ16" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK16" t="s" s="2">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="B17" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="C17" s="2"/>
+      <c r="D17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E17" s="2"/>
+      <c r="F17" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G17" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K17" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="L17" t="s" s="2">
+        <v>30</v>
+      </c>
+      <c r="M17" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="N17" s="2"/>
+      <c r="O17" s="2"/>
+      <c r="P17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q17" s="2"/>
+      <c r="R17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB17" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="AC17" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AD17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE17" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="AF17" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AG17" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH17" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI17" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ17" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK17" t="s" s="2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="2">
+        <v>134</v>
+      </c>
+      <c r="B18" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E18" s="2"/>
+      <c r="F18" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="G18" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K18" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="L18" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="M18" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="N18" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="O18" s="2"/>
+      <c r="P18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q18" s="2"/>
+      <c r="R18" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="S18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF18" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="AG18" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH18" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ18" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK18" t="s" s="2">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="B19" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E19" s="2"/>
+      <c r="F19" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G19" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K19" t="s" s="2">
+        <v>136</v>
+      </c>
+      <c r="L19" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="M19" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="N19" s="2"/>
+      <c r="O19" s="2"/>
+      <c r="P19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q19" s="2"/>
+      <c r="R19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF19" t="s" s="2">
         <v>119</v>
       </c>
-      <c r="AG16" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH16" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AI16" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ16" t="s" s="2">
+      <c r="AG19" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH19" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI19" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ19" t="s" s="2">
         <v>120</v>
       </c>
-      <c r="AK16" t="s" s="2">
+      <c r="AK19" t="s" s="2">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="B20" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E20" s="2"/>
+      <c r="F20" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="G20" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="H20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K20" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="L20" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="M20" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="N20" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="O20" s="2"/>
+      <c r="P20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q20" s="2"/>
+      <c r="R20" t="s" s="2">
+        <v>3</v>
+      </c>
+      <c r="S20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF20" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="AG20" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AH20" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ20" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK20" t="s" s="2">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="B21" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E21" s="2"/>
+      <c r="F21" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G21" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K21" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="L21" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="M21" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="N21" s="2"/>
+      <c r="O21" s="2"/>
+      <c r="P21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q21" s="2"/>
+      <c r="R21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF21" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="AG21" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH21" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AI21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ21" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="AK21" t="s" s="2">
         <v>111</v>
       </c>
     </row>

</xml_diff>